<commit_message>
update: Updated user stories
</commit_message>
<xml_diff>
--- a/user-stories.xlsx
+++ b/user-stories.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/matteo/Library/Mobile Documents/com~apple~CloudDocs/Schule/DBB/2026/HabitQuest/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C56AD977-B9FB-F24A-930E-D9F7E39EEA7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FFAA4CB-B5DA-7643-B86F-4E934289B645}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="19940" xr2:uid="{6E36DC40-5F18-4EBE-9BC3-7D855008A313}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="21380" xr2:uid="{6E36DC40-5F18-4EBE-9BC3-7D855008A313}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="62">
   <si>
     <t>Priority scale</t>
   </si>
@@ -124,9 +124,6 @@
     <t>I get the reward for finishing a habit.</t>
   </si>
   <si>
-    <t>Dynamic experience gian</t>
-  </si>
-  <si>
     <t>gain dynamic amounts of experience - not always the same for the same habit.</t>
   </si>
   <si>
@@ -170,6 +167,76 @@
   </si>
   <si>
     <t>gain rewards by leveling up and finishing habits.</t>
+  </si>
+  <si>
+    <t>User documentation</t>
+  </si>
+  <si>
+    <t>understand the workings of the application and have some form of documentation.</t>
+  </si>
+  <si>
+    <t>in case I get questions about the application, I can always look them up.</t>
+  </si>
+  <si>
+    <t>Product Goal 1 - Basic User Interface</t>
+  </si>
+  <si>
+    <t>Product Goal 2 - Basic Gamification Features</t>
+  </si>
+  <si>
+    <t>Product Goal 3 - Advanced Features</t>
+  </si>
+  <si>
+    <t>Product Goal 4 - User Documentation</t>
+  </si>
+  <si>
+    <t>Dynamic experience gain</t>
+  </si>
+  <si>
+    <t>- The user can create a habit
+- The habit is automatically saved to a database
+- There is a button to select the reoccurance of the habit</t>
+  </si>
+  <si>
+    <t>- When opening the web application the user is in the main window
+- The main window contains space holders for:
+  - Habit creation
+  - The level bar
+  - Current open habits
+  - A switch to toggle between showing all habits and the currently open ones.</t>
+  </si>
+  <si>
+    <t>- All relevant data is loaded from the database
+- All relevant data is displayed in the placeholders
+- The relevant data could be the following
+  - Habits
+  - The current level</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- When completing a habit, the user should be rewarded with Experience points
+- These should be displayed directly when the task is marked as completed. </t>
+  </si>
+  <si>
+    <t>- If the user has accumulated enough experience points, he should level up.</t>
+  </si>
+  <si>
+    <t>- Experience gain should be adjusted over time
+- If a person completes the same habit multiple times in a row, the experience gain should decrease
+- If he ups his goals, he should be rewarded with increased experience gain</t>
+  </si>
+  <si>
+    <t>- The user is able to gain bonus experience if he completes the same habit multiple times in a row, without missing a scheduled habit.</t>
+  </si>
+  <si>
+    <t>- The user can edit a habit that has already been created
+- This can be done through a button in the ui.</t>
+  </si>
+  <si>
+    <t>- The user gets occasional rewards by leveling up
+- These rewards can be displayed in another menu</t>
+  </si>
+  <si>
+    <t>- The documentation contains all files required for the evaluation</t>
   </si>
 </sst>
 </file>
@@ -249,7 +316,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -261,12 +328,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -654,19 +726,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="3:13" x14ac:dyDescent="0.2">
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="F1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="G1" s="7" t="s">
         <v>4</v>
       </c>
       <c r="I1" t="s">
@@ -674,19 +746,19 @@
       </c>
     </row>
     <row r="2" spans="3:13" x14ac:dyDescent="0.2">
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="9">
+      <c r="D2" s="8">
         <v>4</v>
       </c>
-      <c r="E2" s="9">
+      <c r="E2" s="8">
         <v>3</v>
       </c>
-      <c r="F2" s="9">
+      <c r="F2" s="8">
         <v>2</v>
       </c>
-      <c r="G2" s="9">
+      <c r="G2" s="8">
         <v>1</v>
       </c>
       <c r="I2" t="s">
@@ -735,6 +807,9 @@
       <c r="D4" s="5">
         <v>4</v>
       </c>
+      <c r="E4" t="s">
+        <v>47</v>
+      </c>
       <c r="F4" s="5" t="s">
         <v>19</v>
       </c>
@@ -744,23 +819,32 @@
       <c r="H4" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="I4" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="J4" s="5" t="s">
+      <c r="J4" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="K4" s="5"/>
-      <c r="L4" s="5"/>
-      <c r="M4" s="5"/>
-    </row>
-    <row r="5" spans="3:13" ht="64" x14ac:dyDescent="0.2">
+      <c r="K4" s="5">
+        <v>2</v>
+      </c>
+      <c r="L4" s="5">
+        <v>5</v>
+      </c>
+      <c r="M4" s="10" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="3:13" ht="128" x14ac:dyDescent="0.2">
       <c r="C5" s="5" t="s">
         <v>1</v>
       </c>
       <c r="D5" s="5">
         <v>4</v>
       </c>
+      <c r="E5" t="s">
+        <v>47</v>
+      </c>
       <c r="F5" s="5" t="s">
         <v>23</v>
       </c>
@@ -770,25 +854,34 @@
       <c r="H5" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I5" s="5" t="s">
+      <c r="I5" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="J5" s="5" t="s">
+      <c r="J5" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="K5" s="5"/>
-      <c r="L5" s="5"/>
-      <c r="M5" s="6"/>
-    </row>
-    <row r="6" spans="3:13" ht="48" x14ac:dyDescent="0.2">
+      <c r="K5" s="5">
+        <v>13</v>
+      </c>
+      <c r="L5" s="5">
+        <v>31</v>
+      </c>
+      <c r="M5" s="10" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="6" spans="3:13" ht="80" x14ac:dyDescent="0.2">
       <c r="C6" s="5" t="s">
         <v>1</v>
       </c>
       <c r="D6" s="5">
         <v>4</v>
       </c>
+      <c r="E6" t="s">
+        <v>47</v>
+      </c>
       <c r="F6" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G6" s="5">
         <v>3</v>
@@ -796,22 +889,31 @@
       <c r="H6" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I6" s="5" t="s">
+      <c r="I6" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="J6" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="J6" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="K6" s="5"/>
-      <c r="L6" s="5"/>
-      <c r="M6" s="6"/>
-    </row>
-    <row r="7" spans="3:13" ht="32" x14ac:dyDescent="0.2">
+      <c r="K6" s="5">
+        <v>3</v>
+      </c>
+      <c r="L6" s="5">
+        <v>8</v>
+      </c>
+      <c r="M6" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="7" spans="3:13" ht="64" x14ac:dyDescent="0.2">
       <c r="C7" s="5" t="s">
         <v>2</v>
       </c>
       <c r="D7" s="5">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="E7" t="s">
+        <v>48</v>
       </c>
       <c r="F7" s="5" t="s">
         <v>26</v>
@@ -822,25 +924,34 @@
       <c r="H7" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I7" s="5" t="s">
+      <c r="I7" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="J7" s="5" t="s">
+      <c r="J7" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="K7" s="5"/>
-      <c r="L7" s="5"/>
-      <c r="M7" s="7"/>
-    </row>
-    <row r="8" spans="3:13" ht="48" x14ac:dyDescent="0.2">
+      <c r="K7" s="5">
+        <v>3</v>
+      </c>
+      <c r="L7" s="5">
+        <v>8</v>
+      </c>
+      <c r="M7" s="11" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8" spans="3:13" ht="80" x14ac:dyDescent="0.2">
       <c r="C8" s="5" t="s">
         <v>2</v>
       </c>
       <c r="D8" s="5">
         <v>3</v>
       </c>
+      <c r="E8" t="s">
+        <v>49</v>
+      </c>
       <c r="F8" s="5" t="s">
-        <v>29</v>
+        <v>51</v>
       </c>
       <c r="G8" s="5">
         <v>5</v>
@@ -848,15 +959,21 @@
       <c r="H8" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I8" s="5" t="s">
+      <c r="I8" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="J8" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="J8" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="K8" s="5"/>
-      <c r="L8" s="5"/>
-      <c r="M8" s="6"/>
+      <c r="K8" s="5">
+        <v>13</v>
+      </c>
+      <c r="L8" s="5">
+        <v>30</v>
+      </c>
+      <c r="M8" s="10" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="9" spans="3:13" ht="32" x14ac:dyDescent="0.2">
       <c r="C9" s="5" t="s">
@@ -865,8 +982,11 @@
       <c r="D9" s="5">
         <v>4</v>
       </c>
+      <c r="E9" t="s">
+        <v>48</v>
+      </c>
       <c r="F9" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G9" s="5">
         <v>6</v>
@@ -874,15 +994,21 @@
       <c r="H9" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I9" s="5" t="s">
+      <c r="I9" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="J9" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="J9" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="K9" s="5"/>
-      <c r="L9" s="5"/>
-      <c r="M9" s="6"/>
+      <c r="K9" s="5">
+        <v>2</v>
+      </c>
+      <c r="L9" s="5">
+        <v>5</v>
+      </c>
+      <c r="M9" s="10" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="10" spans="3:13" ht="48" x14ac:dyDescent="0.2">
       <c r="C10" s="5" t="s">
@@ -891,8 +1017,11 @@
       <c r="D10" s="5">
         <v>3</v>
       </c>
+      <c r="E10" t="s">
+        <v>49</v>
+      </c>
       <c r="F10" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G10" s="5">
         <v>7</v>
@@ -900,15 +1029,21 @@
       <c r="H10" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I10" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="J10" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5"/>
-      <c r="M10" s="6"/>
+      <c r="I10" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="J10" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="K10" s="5">
+        <v>5</v>
+      </c>
+      <c r="L10" s="5">
+        <v>12</v>
+      </c>
+      <c r="M10" s="10" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="11" spans="3:13" ht="48" x14ac:dyDescent="0.2">
       <c r="C11" s="5" t="s">
@@ -917,8 +1052,11 @@
       <c r="D11" s="5">
         <v>4</v>
       </c>
+      <c r="E11" t="s">
+        <v>47</v>
+      </c>
       <c r="F11" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G11" s="5">
         <v>8</v>
@@ -926,25 +1064,34 @@
       <c r="H11" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I11" s="5" t="s">
+      <c r="I11" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="J11" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="J11" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="K11" s="5"/>
-      <c r="L11" s="5"/>
-      <c r="M11" s="6"/>
+      <c r="K11" s="5">
+        <v>3</v>
+      </c>
+      <c r="L11" s="5">
+        <v>8</v>
+      </c>
+      <c r="M11" s="10" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="12" spans="3:13" ht="32" x14ac:dyDescent="0.2">
       <c r="C12" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D12" s="5">
         <v>3</v>
       </c>
-      <c r="D12" s="5">
-        <v>2</v>
+      <c r="E12" t="s">
+        <v>48</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G12" s="5">
         <v>9</v>
@@ -952,31 +1099,56 @@
       <c r="H12" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I12" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="J12" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="K12" s="5"/>
-      <c r="L12" s="5"/>
-      <c r="M12" s="6"/>
-    </row>
-    <row r="13" spans="3:13" ht="16" x14ac:dyDescent="0.2">
+      <c r="I12" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="J12" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="K12" s="5">
+        <v>8</v>
+      </c>
+      <c r="L12" s="5">
+        <v>20</v>
+      </c>
+      <c r="M12" s="10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="13" spans="3:13" ht="48" x14ac:dyDescent="0.2">
       <c r="C13" s="5" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D13" s="5">
         <v>3</v>
       </c>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5"/>
-      <c r="K13" s="5"/>
-      <c r="L13" s="5"/>
-      <c r="M13" s="6"/>
+      <c r="E13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="G13" s="5">
+        <v>10</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I13" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="J13" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="K13" s="5">
+        <v>13</v>
+      </c>
+      <c r="L13" s="5">
+        <v>30</v>
+      </c>
+      <c r="M13" s="10" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="14" spans="3:13" x14ac:dyDescent="0.2">
       <c r="C14" s="5"/>
@@ -1065,7 +1237,6 @@
     <row r="21" spans="3:13" x14ac:dyDescent="0.2">
       <c r="C21" s="5"/>
       <c r="D21" s="5"/>
-      <c r="E21" s="10"/>
       <c r="F21" s="5"/>
       <c r="G21" s="5"/>
       <c r="H21" s="5"/>
@@ -1078,7 +1249,6 @@
     <row r="22" spans="3:13" x14ac:dyDescent="0.2">
       <c r="C22" s="5"/>
       <c r="D22" s="5"/>
-      <c r="E22" s="10"/>
       <c r="F22" s="5"/>
       <c r="G22" s="5"/>
       <c r="H22" s="5"/>
@@ -1091,7 +1261,6 @@
     <row r="23" spans="3:13" x14ac:dyDescent="0.2">
       <c r="C23" s="5"/>
       <c r="D23" s="5"/>
-      <c r="E23" s="10"/>
       <c r="F23" s="5"/>
       <c r="G23" s="5"/>
       <c r="H23" s="5"/>
@@ -1104,7 +1273,6 @@
     <row r="24" spans="3:13" x14ac:dyDescent="0.2">
       <c r="C24" s="5"/>
       <c r="D24" s="5"/>
-      <c r="E24" s="10"/>
       <c r="F24" s="5"/>
       <c r="G24" s="5"/>
       <c r="H24" s="5"/>
@@ -1117,7 +1285,6 @@
     <row r="25" spans="3:13" x14ac:dyDescent="0.2">
       <c r="C25" s="5"/>
       <c r="D25" s="5"/>
-      <c r="E25" s="10"/>
       <c r="F25" s="5"/>
       <c r="G25" s="5"/>
       <c r="H25" s="5"/>
@@ -1391,18 +1558,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1422,14 +1589,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3CD4954-40DF-4E1B-A417-8AC111E78ABB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BE5B2139-0411-4F93-927B-CEF9303A0586}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -1442,4 +1601,12 @@
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3CD4954-40DF-4E1B-A417-8AC111E78ABB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>